<commit_message>
Atari make file, added new level, inventory finished
</commit_message>
<xml_diff>
--- a/map.xlsx
+++ b/map.xlsx
@@ -16,18 +16,26 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+  <si>
+    <t>9
+LAKE
+monster HP: 3 DEF 3
+TORCH (id:0)</t>
+  </si>
   <si>
     <t>15
-START</t>
+START
+DAGGER (ATT+1)</t>
   </si>
   <si>
-    <t>9
-LAKE</t>
+    <t>14
+THICKED OF BUSHES</t>
   </si>
   <si>
     <t>10
-ISLAND</t>
+ISLAND
+MACHETE (id: 1)</t>
   </si>
 </sst>
 </file>
@@ -140,10 +148,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -443,7 +451,7 @@
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="6" width="18.625" customWidth="1"/>
+    <col min="1" max="6" width="20.625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="80.099999999999994" customHeight="1">
@@ -474,10 +482,10 @@
         <v>8</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2" s="1">
         <v>11</v>
@@ -490,11 +498,11 @@
       <c r="A3" s="1">
         <v>13</v>
       </c>
-      <c r="B3" s="5">
-        <v>14</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>0</v>
+      <c r="B3" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>1</v>
       </c>
       <c r="D3" s="2">
         <v>16</v>

</xml_diff>

<commit_message>
Major refactor, split into files, batch file for creating cp/m disk image
</commit_message>
<xml_diff>
--- a/map.xlsx
+++ b/map.xlsx
@@ -29,13 +29,13 @@
 DAGGER (ATT+1)</t>
   </si>
   <si>
-    <t>14
-THICKED OF BUSHES</t>
-  </si>
-  <si>
     <t>10
 ISLAND
 MACHETE (id: 1)</t>
+  </si>
+  <si>
+    <t>14
+BUSHES</t>
   </si>
 </sst>
 </file>
@@ -485,7 +485,7 @@
         <v>0</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E2" s="1">
         <v>11</v>
@@ -499,7 +499,7 @@
         <v>13</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>1</v>

</xml_diff>

<commit_message>
Refactoring item handling, merge item and weapons handling, automating export for CP/M disk image
</commit_message>
<xml_diff>
--- a/map.xlsx
+++ b/map.xlsx
@@ -16,18 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
-  <si>
-    <t>9
-LAKE
-monster HP: 3 DEF 3
-TORCH (id:0)</t>
-  </si>
-  <si>
-    <t>15
-START
-DAGGER (ATT+1)</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>10
 ISLAND
@@ -36,6 +25,23 @@
   <si>
     <t>14
 BUSHES</t>
+  </si>
+  <si>
+    <t>15
+START
+DAGGER (ATT+1)
+WOODEN SHIELD (DEF + 1)
+POTION</t>
+  </si>
+  <si>
+    <t>9
+LAKE
+MONSTER HP: 3 DEF 3
+TORCH (id:0)</t>
+  </si>
+  <si>
+    <t>STREAM
+20</t>
   </si>
 </sst>
 </file>
@@ -121,10 +127,10 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -451,7 +457,7 @@
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="6" width="20.625" customWidth="1"/>
+    <col min="1" max="6" width="25.625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="80.099999999999994" customHeight="1">
@@ -482,10 +488,10 @@
         <v>8</v>
       </c>
       <c r="C2" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>0</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>2</v>
       </c>
       <c r="E2" s="1">
         <v>11</v>
@@ -498,11 +504,11 @@
       <c r="A3" s="1">
         <v>13</v>
       </c>
-      <c r="B3" s="6" t="s">
-        <v>3</v>
+      <c r="B3" s="4" t="s">
+        <v>1</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D3" s="2">
         <v>16</v>
@@ -518,8 +524,8 @@
       <c r="A4" s="1">
         <v>19</v>
       </c>
-      <c r="B4" s="1">
-        <v>20</v>
+      <c r="B4" s="6" t="s">
+        <v>4</v>
       </c>
       <c r="C4" s="1">
         <v>21</v>

</xml_diff>

<commit_message>
Optimalisation of reading keys, new locations, new weapon
</commit_message>
<xml_diff>
--- a/map.xlsx
+++ b/map.xlsx
@@ -16,16 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
-  <si>
-    <t>10
-ISLAND
-MACHETE (id: 1)</t>
-  </si>
-  <si>
-    <t>14
-BUSHES</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>15
 START
@@ -34,14 +25,39 @@
 POTION</t>
   </si>
   <si>
+    <t>STREAM
+20</t>
+  </si>
+  <si>
+    <t>14
+BUSHES
+(potrzeba maczety, żeby przejść)</t>
+  </si>
+  <si>
+    <t>10
+ISLAND
+(potrzeba pochodni żeby coś zobaczyć) MACHETE (id: 1)</t>
+  </si>
+  <si>
     <t>9
 LAKE
-MONSTER HP: 3 DEF 3
-TORCH (id:0)</t>
-  </si>
-  <si>
-    <t>STREAM
-20</t>
+MONSTER HP: 5 DEF 3
+(po pokonaniu potwora wypada pochodnia - TORCH id:0)</t>
+  </si>
+  <si>
+    <t>27
+ROCKS</t>
+  </si>
+  <si>
+    <t>26
+SPRING
+MONSTER HP: 9 DEF 5
+(po pokonaniu potwora wypada POTION i pozwala przejść do E)</t>
+  </si>
+  <si>
+    <t>CAVE
+SHORT SWORD (ATT +3)
+21</t>
   </si>
 </sst>
 </file>
@@ -65,7 +81,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -131,16 +147,38 @@
         <color indexed="64"/>
       </right>
       <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -158,6 +196,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -460,7 +504,7 @@
     <col min="1" max="6" width="25.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="80.099999999999994" customHeight="1">
+    <row r="1" spans="1:6" ht="90" customHeight="1">
       <c r="A1" s="1">
         <v>1</v>
       </c>
@@ -480,7 +524,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="80.099999999999994" customHeight="1">
+    <row r="2" spans="1:6" ht="90" customHeight="1">
       <c r="A2" s="1">
         <v>7</v>
       </c>
@@ -488,10 +532,10 @@
         <v>8</v>
       </c>
       <c r="C2" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>3</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>0</v>
       </c>
       <c r="E2" s="1">
         <v>11</v>
@@ -500,15 +544,15 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="80.099999999999994" customHeight="1">
+    <row r="3" spans="1:6" ht="90" customHeight="1">
       <c r="A3" s="1">
         <v>13</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D3" s="2">
         <v>16</v>
@@ -520,15 +564,15 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="80.099999999999994" customHeight="1">
+    <row r="4" spans="1:6" ht="90" customHeight="1">
       <c r="A4" s="1">
         <v>19</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="1">
-        <v>21</v>
+        <v>1</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>7</v>
       </c>
       <c r="D4" s="1">
         <v>22</v>
@@ -540,15 +584,15 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="80.099999999999994" customHeight="1">
+    <row r="5" spans="1:6" ht="90" customHeight="1">
       <c r="A5" s="1">
         <v>25</v>
       </c>
-      <c r="B5" s="1">
-        <v>26</v>
-      </c>
-      <c r="C5" s="1">
-        <v>27</v>
+      <c r="B5" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>5</v>
       </c>
       <c r="D5" s="1">
         <v>28</v>
@@ -560,7 +604,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="80.099999999999994" customHeight="1">
+    <row r="6" spans="1:6" ht="90" customHeight="1">
       <c r="A6" s="1">
         <v>31</v>
       </c>

</xml_diff>

<commit_message>
New locations, updated cp/m transfer make file, rewritten item management
</commit_message>
<xml_diff>
--- a/map.xlsx
+++ b/map.xlsx
@@ -55,9 +55,10 @@
 (po pokonaniu potwora wypada POTION i pozwala przejść do E)</t>
   </si>
   <si>
-    <t>CAVE
+    <t>21
+CAVE
 SHORT SWORD (ATT +3)
-21</t>
+PERUN'S STONE</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
New locations, new weapons, expanded descriptions
</commit_message>
<xml_diff>
--- a/map.xlsx
+++ b/map.xlsx
@@ -8,15 +8,13 @@
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
-    <sheet name="Arkusz2" sheetId="2" r:id="rId2"/>
-    <sheet name="Arkusz3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>15
 START
@@ -25,10 +23,6 @@
 POTION</t>
   </si>
   <si>
-    <t>STREAM
-20</t>
-  </si>
-  <si>
     <t>14
 BUSHES
 (potrzeba maczety, żeby przejść)</t>
@@ -59,6 +53,19 @@
 CAVE
 SHORT SWORD (ATT +3)
 PERUN'S STONE</t>
+  </si>
+  <si>
+    <t>20
+STREAM</t>
+  </si>
+  <si>
+    <t>19
+FOREST_1
+BIES HP 6, DEF 2</t>
+  </si>
+  <si>
+    <t>25
+FOREST_2</t>
   </si>
 </sst>
 </file>
@@ -82,7 +89,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -144,6 +151,28 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -155,31 +184,20 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
       <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -203,6 +221,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -533,10 +554,10 @@
         <v>8</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E2" s="1">
         <v>11</v>
@@ -550,7 +571,7 @@
         <v>13</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>0</v>
@@ -566,14 +587,14 @@
       </c>
     </row>
     <row r="4" spans="1:6" ht="90" customHeight="1">
-      <c r="A4" s="1">
-        <v>19</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="8" t="s">
+      <c r="A4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="8" t="s">
         <v>7</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>6</v>
       </c>
       <c r="D4" s="1">
         <v>22</v>
@@ -586,14 +607,14 @@
       </c>
     </row>
     <row r="5" spans="1:6" ht="90" customHeight="1">
-      <c r="A5" s="1">
-        <v>25</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>6</v>
+      <c r="A5" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>5</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D5" s="1">
         <v>28</v>
@@ -629,22 +650,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Split locations into separate files, new monsters and locations.
</commit_message>
<xml_diff>
--- a/map.xlsx
+++ b/map.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>15
 START
@@ -33,20 +33,8 @@
 (potrzeba pochodni żeby coś zobaczyć) MACHETE (id: 1)</t>
   </si>
   <si>
-    <t>9
-LAKE
-MONSTER HP: 5 DEF 3
-(po pokonaniu potwora wypada pochodnia - TORCH id:0)</t>
-  </si>
-  <si>
     <t>27
 ROCKS</t>
-  </si>
-  <si>
-    <t>26
-SPRING
-MONSTER HP: 9 DEF 5
-(po pokonaniu potwora wypada POTION i pozwala przejść do E)</t>
   </si>
   <si>
     <t>21
@@ -59,13 +47,38 @@
 STREAM</t>
   </si>
   <si>
+    <t>25
+FOREST_2</t>
+  </si>
+  <si>
+    <t>31
+FOREST_3</t>
+  </si>
+  <si>
+    <t>33
+THE_LESHY_VALLEY</t>
+  </si>
+  <si>
+    <t>32
+SVAROG_STONE_CIRCLE
+LESHY HP 15 DEF 4 ATT 8</t>
+  </si>
+  <si>
+    <t>26
+SPRING
+MONSTER HP 9 DEF 5 ATT 9
+(po pokonaniu potwora wypada POTION i pozwala przejść do E)</t>
+  </si>
+  <si>
+    <t>9
+LAKE
+MONSTER HP 5 DEF 3 ATT 5
+(po pokonaniu potwora wypada pochodnia - TORCH id:0)</t>
+  </si>
+  <si>
     <t>19
 FOREST_1
-BIES HP 6, DEF 2</t>
-  </si>
-  <si>
-    <t>25
-FOREST_2</t>
+BIES HP 6, DEF 2 ATT 2</t>
   </si>
 </sst>
 </file>
@@ -89,7 +102,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -188,6 +201,15 @@
         <color indexed="64"/>
       </right>
       <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -197,7 +219,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -223,7 +245,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -554,7 +579,7 @@
         <v>8</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>2</v>
@@ -588,13 +613,13 @@
     </row>
     <row r="4" spans="1:6" ht="90" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D4" s="1">
         <v>22</v>
@@ -608,13 +633,13 @@
     </row>
     <row r="5" spans="1:6" ht="90" customHeight="1">
       <c r="A5" s="9" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D5" s="1">
         <v>28</v>
@@ -627,14 +652,14 @@
       </c>
     </row>
     <row r="6" spans="1:6" ht="90" customHeight="1">
-      <c r="A6" s="1">
-        <v>31</v>
-      </c>
-      <c r="B6" s="1">
-        <v>32</v>
-      </c>
-      <c r="C6" s="1">
-        <v>33</v>
+      <c r="A6" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>8</v>
       </c>
       <c r="D6" s="1">
         <v>34</v>

</xml_diff>

<commit_message>
New locations, new weapons
</commit_message>
<xml_diff>
--- a/map.xlsx
+++ b/map.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>15
 START
@@ -79,6 +79,21 @@
     <t>19
 FOREST_1
 BIES HP 6, DEF 2 ATT 2</t>
+  </si>
+  <si>
+    <t>13
+GOLDEN_FIELD
+BUTY +1</t>
+  </si>
+  <si>
+    <t>7
+STONE_THRESHOLD</t>
+  </si>
+  <si>
+    <t>1
+SACRED_GROVE
+PLANETNIK HP 10, DEF 5, ATT 5
+(po pokonaniu potwora wypada kamień do tarczy - Stone of Dzivogon id:50)</t>
   </si>
 </sst>
 </file>
@@ -102,7 +117,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -215,11 +230,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -249,6 +273,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -551,9 +581,9 @@
     <col min="1" max="6" width="25.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="90" customHeight="1">
-      <c r="A1" s="1">
-        <v>1</v>
+    <row r="1" spans="1:6" ht="99.95" customHeight="1">
+      <c r="A1" s="7" t="s">
+        <v>15</v>
       </c>
       <c r="B1" s="1">
         <v>2</v>
@@ -571,9 +601,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="90" customHeight="1">
-      <c r="A2" s="1">
-        <v>7</v>
+    <row r="2" spans="1:6" ht="99.95" customHeight="1">
+      <c r="A2" s="12" t="s">
+        <v>14</v>
       </c>
       <c r="B2" s="1">
         <v>8</v>
@@ -591,8 +621,8 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="90" customHeight="1">
-      <c r="A3" s="1">
+    <row r="3" spans="1:6" ht="99.95" customHeight="1">
+      <c r="A3" s="12" t="s">
         <v>13</v>
       </c>
       <c r="B3" s="4" t="s">
@@ -611,8 +641,8 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="90" customHeight="1">
-      <c r="A4" s="4" t="s">
+    <row r="4" spans="1:6" ht="99.95" customHeight="1">
+      <c r="A4" s="11" t="s">
         <v>12</v>
       </c>
       <c r="B4" s="8" t="s">
@@ -631,7 +661,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="90" customHeight="1">
+    <row r="5" spans="1:6" ht="99.95" customHeight="1">
       <c r="A5" s="9" t="s">
         <v>6</v>
       </c>
@@ -651,7 +681,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="90" customHeight="1">
+    <row r="6" spans="1:6" ht="99.95" customHeight="1">
       <c r="A6" s="6" t="s">
         <v>7</v>
       </c>

</xml_diff>

<commit_message>
Default key reading optimised, new items, fix for magic stones
</commit_message>
<xml_diff>
--- a/map.xlsx
+++ b/map.xlsx
@@ -55,15 +55,6 @@
 FOREST_3</t>
   </si>
   <si>
-    <t>33
-THE_LESHY_VALLEY</t>
-  </si>
-  <si>
-    <t>32
-SVAROG_STONE_CIRCLE
-LESHY HP 15 DEF 4 ATT 8</t>
-  </si>
-  <si>
     <t>26
 SPRING
 MONSTER HP 9 DEF 5 ATT 9
@@ -90,10 +81,21 @@
 STONE_THRESHOLD</t>
   </si>
   <si>
+    <t>32
+SVAROG_STONE_CIRCLE
+LESHY HP 15 DEF 4 ATT 8
+(po pokonaniu potwora wypada kamień do broni - Bronze stone id:40)</t>
+  </si>
+  <si>
     <t>1
 SACRED_GROVE
 PLANETNIK HP 10, DEF 5, ATT 5
-(po pokonaniu potwora wypada kamień do tarczy - Stone of Dzivogon id:50)</t>
+(po pokonaniu potwora wypada kamień do tarczy - Stone of Dzivogon id:50 oraz BONDCUTTER konieczny w 33)</t>
+  </si>
+  <si>
+    <t>33
+THE_LESHY_VALLEY
+(potrzeba BONDCUTTER, żeby przejść dalej)</t>
   </si>
 </sst>
 </file>
@@ -578,12 +580,12 @@
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="6" width="25.625" customWidth="1"/>
+    <col min="1" max="6" width="30.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="99.95" customHeight="1">
+    <row r="1" spans="1:6" ht="105.75" customHeight="1">
       <c r="A1" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B1" s="1">
         <v>2</v>
@@ -603,13 +605,13 @@
     </row>
     <row r="2" spans="1:6" ht="99.95" customHeight="1">
       <c r="A2" s="12" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B2" s="1">
         <v>8</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>2</v>
@@ -623,7 +625,7 @@
     </row>
     <row r="3" spans="1:6" ht="99.95" customHeight="1">
       <c r="A3" s="12" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>1</v>
@@ -643,7 +645,7 @@
     </row>
     <row r="4" spans="1:6" ht="99.95" customHeight="1">
       <c r="A4" s="11" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>5</v>
@@ -666,7 +668,7 @@
         <v>6</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>3</v>
@@ -686,12 +688,12 @@
         <v>7</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D6" s="1">
+        <v>13</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="2">
         <v>34</v>
       </c>
       <c r="E6" s="1">

</xml_diff>

<commit_message>
New locations, bug fixes for drop items, new items, new procedure for potential text wrapping
</commit_message>
<xml_diff>
--- a/map.xlsx
+++ b/map.xlsx
@@ -14,14 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
-  <si>
-    <t>15
-START
-DAGGER (ATT+1)
-WOODEN SHIELD (DEF + 1)
-POTION</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>14
 BUSHES
@@ -37,12 +30,6 @@
 ROCKS</t>
   </si>
   <si>
-    <t>21
-CAVE
-SHORT SWORD (ATT +3)
-PERUN'S STONE</t>
-  </si>
-  <si>
     <t>20
 STREAM</t>
   </si>
@@ -53,12 +40,6 @@
   <si>
     <t>31
 FOREST_3</t>
-  </si>
-  <si>
-    <t>26
-SPRING
-MONSTER HP 9 DEF 5 ATT 9
-(po pokonaniu potwora wypada POTION i pozwala przejść do E)</t>
   </si>
   <si>
     <t>9
@@ -72,19 +53,8 @@
 BIES HP 6, DEF 2 ATT 2</t>
   </si>
   <si>
-    <t>13
-GOLDEN_FIELD
-BUTY +1</t>
-  </si>
-  <si>
     <t>7
 STONE_THRESHOLD</t>
-  </si>
-  <si>
-    <t>32
-SVAROG_STONE_CIRCLE
-LESHY HP 15 DEF 4 ATT 8
-(po pokonaniu potwora wypada kamień do broni - Bronze stone id:40)</t>
   </si>
   <si>
     <t>1
@@ -96,18 +66,100 @@
     <t>33
 THE_LESHY_VALLEY
 (potrzeba BONDCUTTER, żeby przejść dalej)</t>
+  </si>
+  <si>
+    <t>34
+LAKE_NIGHT_DAY
+CLOAK OF WELLES</t>
+  </si>
+  <si>
+    <t>26
+SPRING
+STRIGA HP 9 DEF 5 ATT 9
+(po pokonaniu potwora wypada POTION i pozwala przejść do E)</t>
+  </si>
+  <si>
+    <t>15
+START
+NIGHT THORN (ATT+1)
+WOODEN SHIELD (DEF + 1)
+POTION</t>
+  </si>
+  <si>
+    <t>32
+SVAROG_STONE_CIRCLE
+LESHY HP 15 DEF 4 ATT 8
+(po pokonaniu potwora wypada kamień do broni - BRONZE STONE id:40)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">21
+CAVE
+BLOOD_HARVEST (ATT +3)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>PERUN'S STONE</t>
+    </r>
+  </si>
+  <si>
+    <t>13
+GOLDEN_FIELD
+WINGS_OF_THE_WIND +1</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">28
+LOCATION_MORANA_CIRCLE
+MORANA HP 15 DEF 7 ATT 6
+(po pokonaniu wypada </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>SVAROG'S HAMMER</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve"> i Iron Stronghold)</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Czcionka tekstu podstawowego"/>
       <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Czcionka tekstu podstawowego"/>
       <charset val="238"/>
     </font>
   </fonts>
@@ -585,7 +637,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="105.75" customHeight="1">
       <c r="A1" s="7" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="B1" s="1">
         <v>2</v>
@@ -605,16 +657,16 @@
     </row>
     <row r="2" spans="1:6" ht="99.95" customHeight="1">
       <c r="A2" s="12" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B2" s="1">
         <v>8</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E2" s="1">
         <v>11</v>
@@ -625,13 +677,13 @@
     </row>
     <row r="3" spans="1:6" ht="99.95" customHeight="1">
       <c r="A3" s="12" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="D3" s="2">
         <v>16</v>
@@ -645,13 +697,13 @@
     </row>
     <row r="4" spans="1:6" ht="99.95" customHeight="1">
       <c r="A4" s="11" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="D4" s="1">
         <v>22</v>
@@ -665,16 +717,16 @@
     </row>
     <row r="5" spans="1:6" ht="99.95" customHeight="1">
       <c r="A5" s="9" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="D5" s="1">
-        <v>28</v>
+        <v>2</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="E5" s="1">
         <v>29</v>
@@ -685,16 +737,16 @@
     </row>
     <row r="6" spans="1:6" ht="99.95" customHeight="1">
       <c r="A6" s="6" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" s="2">
-        <v>34</v>
+        <v>10</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>11</v>
       </c>
       <c r="E6" s="1">
         <v>35</v>

</xml_diff>

<commit_message>
New locations, configuration moved to external app.
</commit_message>
<xml_diff>
--- a/map.xlsx
+++ b/map.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>14
 BUSHES
@@ -141,6 +141,15 @@
       </rPr>
       <t xml:space="preserve"> i Iron Stronghold)</t>
     </r>
+  </si>
+  <si>
+    <t>22
+MOUND</t>
+  </si>
+  <si>
+    <t>16
+MOUND_INSIDE
+NIGHT_PREACHER HP 20, DEF 9, ATT 8 (po pokonaniu potwora wypada HEAD_SOUTHERN_SUN)</t>
   </si>
 </sst>
 </file>
@@ -297,12 +306,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
@@ -636,7 +642,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="105.75" customHeight="1">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="6" t="s">
         <v>9</v>
       </c>
       <c r="B1" s="1">
@@ -656,16 +662,16 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="99.95" customHeight="1">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="11" t="s">
         <v>8</v>
       </c>
       <c r="B2" s="1">
         <v>8</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>1</v>
       </c>
       <c r="E2" s="1">
@@ -676,17 +682,17 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="99.95" customHeight="1">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="2">
-        <v>16</v>
+      <c r="D3" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="E3" s="1">
         <v>17</v>
@@ -696,17 +702,17 @@
       </c>
     </row>
     <row r="4" spans="1:6" ht="99.95" customHeight="1">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="1">
-        <v>22</v>
+      <c r="D4" s="11" t="s">
+        <v>18</v>
       </c>
       <c r="E4" s="1">
         <v>23</v>
@@ -716,16 +722,16 @@
       </c>
     </row>
     <row r="5" spans="1:6" ht="99.95" customHeight="1">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="11" t="s">
         <v>17</v>
       </c>
       <c r="E5" s="1">
@@ -736,16 +742,16 @@
       </c>
     </row>
     <row r="6" spans="1:6" ht="99.95" customHeight="1">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="4" t="s">
         <v>11</v>
       </c>
       <c r="E6" s="1">

</xml_diff>

<commit_message>
New locations, new items
</commit_message>
<xml_diff>
--- a/map.xlsx
+++ b/map.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>14
 BUSHES
@@ -147,9 +147,19 @@
 MOUND</t>
   </si>
   <si>
+    <t>23
+WIND_AND_BONE_PASS
+POTION</t>
+  </si>
+  <si>
+    <t>29
+LAKE_OF_SOULS
+(potrzeba BONE TOKEN żeby przejść dalej)</t>
+  </si>
+  <si>
     <t>16
 MOUND_INSIDE
-NIGHT_PREACHER HP 20, DEF 9, ATT 8 (po pokonaniu potwora wypada HEAD_SOUTHERN_SUN)</t>
+NIGHT_PREACHER HP 20, DEF 9, ATT 8 (po pokonaniu potwora wypada HEAD_SOUTHERN_SUN i BONE TOKEN)</t>
   </si>
 </sst>
 </file>
@@ -180,7 +190,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -302,11 +312,35 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -339,6 +373,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -692,7 +732,7 @@
         <v>13</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E3" s="1">
         <v>17</v>
@@ -711,11 +751,11 @@
       <c r="C4" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="1">
-        <v>23</v>
+      <c r="E4" s="12" t="s">
+        <v>19</v>
       </c>
       <c r="F4" s="1">
         <v>24</v>
@@ -734,8 +774,8 @@
       <c r="D5" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="1">
-        <v>29</v>
+      <c r="E5" s="13" t="s">
+        <v>20</v>
       </c>
       <c r="F5" s="1">
         <v>30</v>

</xml_diff>

<commit_message>
New location, new terminal added to configuration app, clear screen escape code added (BOSMAN not tested)
</commit_message>
<xml_diff>
--- a/map.xlsx
+++ b/map.xlsx
@@ -14,18 +14,13 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>14
 BUSHES
 (potrzeba maczety, żeby przejść)</t>
   </si>
   <si>
-    <t>10
-ISLAND
-(potrzeba pochodni żeby coś zobaczyć) MACHETE (id: 1)</t>
-  </si>
-  <si>
     <t>27
 ROCKS</t>
   </si>
@@ -42,25 +37,8 @@
 FOREST_3</t>
   </si>
   <si>
-    <t>9
-LAKE
-MONSTER HP 5 DEF 3 ATT 5
-(po pokonaniu potwora wypada pochodnia - TORCH id:0)</t>
-  </si>
-  <si>
-    <t>19
-FOREST_1
-BIES HP 6, DEF 2 ATT 2</t>
-  </si>
-  <si>
     <t>7
 STONE_THRESHOLD</t>
-  </si>
-  <si>
-    <t>1
-SACRED_GROVE
-PLANETNIK HP 10, DEF 5, ATT 5
-(po pokonaniu potwora wypada kamień do tarczy - Stone of Dzivogon id:50 oraz BONDCUTTER konieczny w 33)</t>
   </si>
   <si>
     <t>33
@@ -68,88 +46,8 @@
 (potrzeba BONDCUTTER, żeby przejść dalej)</t>
   </si>
   <si>
-    <t>34
-LAKE_NIGHT_DAY
-CLOAK OF WELLES</t>
-  </si>
-  <si>
-    <t>26
-SPRING
-STRIGA HP 9 DEF 5 ATT 9
-(po pokonaniu potwora wypada POTION i pozwala przejść do E)</t>
-  </si>
-  <si>
-    <t>15
-START
-NIGHT THORN (ATT+1)
-WOODEN SHIELD (DEF + 1)
-POTION</t>
-  </si>
-  <si>
-    <t>32
-SVAROG_STONE_CIRCLE
-LESHY HP 15 DEF 4 ATT 8
-(po pokonaniu potwora wypada kamień do broni - BRONZE STONE id:40)</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">21
-CAVE
-BLOOD_HARVEST (ATT +3)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Czcionka tekstu podstawowego"/>
-        <charset val="238"/>
-      </rPr>
-      <t>PERUN'S STONE</t>
-    </r>
-  </si>
-  <si>
-    <t>13
-GOLDEN_FIELD
-WINGS_OF_THE_WIND +1</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">28
-LOCATION_MORANA_CIRCLE
-MORANA HP 15 DEF 7 ATT 6
-(po pokonaniu wypada </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Czcionka tekstu podstawowego"/>
-        <charset val="238"/>
-      </rPr>
-      <t>SVAROG'S HAMMER</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Czcionka tekstu podstawowego"/>
-        <family val="2"/>
-        <charset val="238"/>
-      </rPr>
-      <t xml:space="preserve"> i Iron Stronghold)</t>
-    </r>
-  </si>
-  <si>
     <t>22
 MOUND</t>
-  </si>
-  <si>
-    <t>23
-WIND_AND_BONE_PASS
-POTION</t>
   </si>
   <si>
     <t>29
@@ -157,24 +55,543 @@
 (potrzeba BONE TOKEN żeby przejść dalej)</t>
   </si>
   <si>
-    <t>16
-MOUND_INSIDE
-NIGHT_PREACHER HP 20, DEF 9, ATT 8 (po pokonaniu potwora wypada HEAD_SOUTHERN_SUN i BONE TOKEN)</t>
-  </si>
-  <si>
     <t>35
 DARK_HARBOUR</t>
   </si>
   <si>
     <t>36
 BLOODY_ROOTS</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">13
+GOLDEN_FIELD
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>WINGS_OF_THE_WIND</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve"> +1</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">34
+LAKE_NIGHT_DAY
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>CLOAK OF WELLES</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">10
+ISLAND
+(potrzeba pochodni żeby coś zobaczyć) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="3" tint="0.39997558519241921"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>MACHETE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve"> (id: 1)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">15
+START
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>NIGHT THORN (ATT+1)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>WOODEN SHIELD (DEF + 1)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="3" tint="0.39997558519241921"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>POTION</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">23
+WIND_AND_BONE_PASS
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="3" tint="0.39997558519241921"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>POTION</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">17
+LOCATION_ECHOES
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="3" tint="0.39997558519241921"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>BONE_TOKEN</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1
+SACRED_GROVE
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>PLANETNIK HP 10, DEF 5, ATT 5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve">
+(po pokonaniu potwora wypada kamień do tarczy - </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>STONE OF DZIVOGON</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve"> id:50 oraz </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="3" tint="0.39997558519241921"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>BONDCUTTER</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve"> konieczny w 33)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">19
+FOREST_1
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>BIES HP 6, DEF 2 ATT 2</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">9
+LAKE
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>DROWNER HP 5 DEF 3 ATT 5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve">
+(po pokonaniu potwora wypada pochodnia - </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="3" tint="0.39997558519241921"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>TORCH</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve"> id:0)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">16
+MOUND_INSIDE
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>NIGHT PREACHER HP 20, DEF 9, ATT 8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve"> (po pokonaniu potwora wypada </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>HEAD_SOUTHERN_SUN</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>)
+potrzeba pochodni, żeby przejść E</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">26
+SPRING
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>STRIGA HP 9 DEF 5 ATT 9</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve">
+(po pokonaniu potwora wypada </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="3" tint="0.39997558519241921"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>POTION</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve"> i pozwala przejść do E)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">32
+SVAROG_STONE_CIRCLE
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>LESHY HP 15 DEF 4 ATT 8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve">
+(po pokonaniu potwora wypada kamień do broni - </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>BRONZE STONE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve"> id:40)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">21
+CAVE
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>BLOOD_HARVEST (ATT +3)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>PERUN'S STONE</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">28
+LOCATION_MORANA_CIRCLE
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>MORANA HP 15 DEF 7 ATT 6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve">
+(po pokonaniu wypada </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>SVAROG'S HAMMER</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve"> i </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>IRON_STRONGOLD</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>)</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -183,9 +600,27 @@
       <charset val="238"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="9" tint="-0.249977111117893"/>
+      <name val="Czcionka tekstu podstawowego"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="3" tint="0.39997558519241921"/>
+      <name val="Czcionka tekstu podstawowego"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Czcionka tekstu podstawowego"/>
+      <charset val="238"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF0070C0"/>
       <name val="Czcionka tekstu podstawowego"/>
       <charset val="238"/>
     </font>
@@ -198,7 +633,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -210,26 +645,33 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
+      <right/>
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin">
+      <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -238,51 +680,7 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
+      <right style="medium">
         <color indexed="64"/>
       </right>
       <top/>
@@ -290,10 +688,30 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <left style="medium">
         <color indexed="64"/>
       </left>
-      <right style="thin">
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
         <color indexed="64"/>
       </right>
       <top/>
@@ -302,11 +720,13 @@
     </border>
     <border>
       <left/>
-      <right/>
-      <top style="thin">
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -317,18 +737,18 @@
       </left>
       <right/>
       <top/>
-      <bottom/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -338,15 +758,21 @@
   <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
@@ -358,9 +784,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -368,9 +791,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -670,127 +1090,127 @@
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="6" width="30.625" customWidth="1"/>
+    <col min="1" max="6" width="35.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="105.75" customHeight="1">
-      <c r="A1" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B1" s="1">
+    <row r="1" spans="1:6" ht="105.75" customHeight="1" thickBot="1">
+      <c r="A1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="4">
         <v>2</v>
       </c>
-      <c r="C1" s="1">
+      <c r="C1" s="4">
         <v>3</v>
       </c>
-      <c r="D1" s="1">
+      <c r="D1" s="4">
         <v>4</v>
       </c>
-      <c r="E1" s="1">
+      <c r="E1" s="4">
         <v>5</v>
       </c>
-      <c r="F1" s="1">
+      <c r="F1" s="4">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="99.95" customHeight="1">
-      <c r="A2" s="11" t="s">
+    <row r="2" spans="1:6" ht="99.95" customHeight="1" thickBot="1">
+      <c r="A2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="4">
         <v>8</v>
       </c>
-      <c r="B2" s="1">
-        <v>8</v>
-      </c>
       <c r="C2" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2" s="1">
+        <v>19</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="4">
         <v>11</v>
       </c>
-      <c r="F2" s="1">
+      <c r="F2" s="4">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="99.95" customHeight="1">
-      <c r="A3" s="11" t="s">
-        <v>16</v>
+    <row r="3" spans="1:6" ht="99.95" customHeight="1" thickBot="1">
+      <c r="A3" s="5" t="s">
+        <v>11</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" s="6" t="s">
+      <c r="C3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="4">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="99.95" customHeight="1" thickBot="1">
+      <c r="A4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="4">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="99.95" customHeight="1" thickBot="1">
+      <c r="A5" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="E3" s="1">
-        <v>17</v>
-      </c>
-      <c r="F3" s="1">
-        <v>18</v>
+      <c r="C5" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" s="4">
+        <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="99.95" customHeight="1">
-      <c r="A4" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="F4" s="1">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="99.95" customHeight="1">
-      <c r="A5" s="8" t="s">
+    <row r="6" spans="1:6" ht="99.95" customHeight="1" thickBot="1">
+      <c r="A6" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B6" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D5" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="F5" s="1">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="99.95" customHeight="1">
-      <c r="A6" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="9" t="s">
+      <c r="E6" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6" s="12" t="s">
         <v>10</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
New locations, new weapons and items, added error handling in configuration app, bug fixes.
</commit_message>
<xml_diff>
--- a/map.xlsx
+++ b/map.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>14
 BUSHES
@@ -37,10 +37,6 @@
 FOREST_3</t>
   </si>
   <si>
-    <t>7
-STONE_THRESHOLD</t>
-  </si>
-  <si>
     <t>33
 THE_LESHY_VALLEY
 (potrzeba BONDCUTTER, żeby przejść dalej)</t>
@@ -64,6 +60,235 @@
   </si>
   <si>
     <r>
+      <t xml:space="preserve">19
+FOREST_1
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>BIES HP 6, DEF 2 ATT 2</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">16
+MOUND_INSIDE
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>NIGHT PREACHER HP 20, DEF 9, ATT 8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve"> (po pokonaniu potwora wypada </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>HEAD_SOUTHERN_SUN</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>)
+potrzeba pochodni, żeby przejść E</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">21
+CAVE
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>WEAPON_BLOOD_HARVEST (ATT +3)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>PERUN'S STONE</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">28
+LOCATION_MORANA_CIRCLE
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>MORANA HP 15 DEF 7 ATT 6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve">
+(po pokonaniu wypada 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>SVAROG'S HAMMER</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>SHIELD_IRON_STRONGOLD</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">34
+LAKE_NIGHT_DAY
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>BODY_CLOAK OF WELLES</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">32
+SVAROG_STONE_CIRCLE
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>LESHY HP 15 DEF 4 ATT 8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve">
+(po pokonaniu potwora wypada kamień do broni - </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>WEAPON_BRONZE_STONE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <r>
       <t xml:space="preserve">13
 GOLDEN_FIELD
 </t>
@@ -75,33 +300,53 @@
         <rFont val="Czcionka tekstu podstawowego"/>
         <charset val="238"/>
       </rPr>
-      <t>WINGS_OF_THE_WIND</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Czcionka tekstu podstawowego"/>
-        <family val="2"/>
-        <charset val="238"/>
-      </rPr>
-      <t xml:space="preserve"> +1</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">34
-LAKE_NIGHT_DAY
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="9" tint="-0.249977111117893"/>
-        <rFont val="Czcionka tekstu podstawowego"/>
-        <charset val="238"/>
-      </rPr>
-      <t>CLOAK OF WELLES</t>
+      <t>BOOTS_WINGS_OF_THE_WIND</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">9
+LAKE
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>DROWNER HP 5 DEF 3 ATT 5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve">
+(po pokonaniu potwora wypada pochodnia - </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="3" tint="0.39997558519241921"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ITEM_TORCH</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>)</t>
     </r>
   </si>
   <si>
@@ -117,7 +362,7 @@
         <rFont val="Czcionka tekstu podstawowego"/>
         <charset val="238"/>
       </rPr>
-      <t>MACHETE</t>
+      <t>ITEM_MACHETE</t>
     </r>
     <r>
       <rPr>
@@ -128,6 +373,94 @@
         <charset val="238"/>
       </rPr>
       <t xml:space="preserve"> (id: 1)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">17
+LOCATION_ECHOES
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="3" tint="0.39997558519241921"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve">ITEM_BONE_TOKEN
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>SHIELD_JAROVITS_BEDROCK</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">23
+WIND_AND_BONE_PASS
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="3" tint="0.39997558519241921"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ITEM_POTION</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">26
+SPRING
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>STRIGA HP 9 DEF 5 ATT 9</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve">
+(po pokonaniu potwora wypada </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="3" tint="0.39997558519241921"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ITEM_POTION</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve"> i pozwala przejść do E)</t>
     </r>
   </si>
   <si>
@@ -143,7 +476,7 @@
         <rFont val="Czcionka tekstu podstawowego"/>
         <charset val="238"/>
       </rPr>
-      <t>NIGHT THORN (ATT+1)</t>
+      <t>WEAPON_NIGHT THORN (ATT+1)</t>
     </r>
     <r>
       <rPr>
@@ -163,7 +496,7 @@
         <rFont val="Czcionka tekstu podstawowego"/>
         <charset val="238"/>
       </rPr>
-      <t>WOODEN SHIELD (DEF + 1)</t>
+      <t>SHIELD_WOODEN SHIELD (DEF + 1)</t>
     </r>
     <r>
       <rPr>
@@ -183,39 +516,7 @@
         <rFont val="Czcionka tekstu podstawowego"/>
         <charset val="238"/>
       </rPr>
-      <t>POTION</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">23
-WIND_AND_BONE_PASS
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="3" tint="0.39997558519241921"/>
-        <rFont val="Czcionka tekstu podstawowego"/>
-        <charset val="238"/>
-      </rPr>
-      <t>POTION</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">17
-LOCATION_ECHOES
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="3" tint="0.39997558519241921"/>
-        <rFont val="Czcionka tekstu podstawowego"/>
-        <charset val="238"/>
-      </rPr>
-      <t>BONE_TOKEN</t>
+      <t>ITEM_POTION</t>
     </r>
   </si>
   <si>
@@ -251,17 +552,17 @@
         <rFont val="Czcionka tekstu podstawowego"/>
         <charset val="238"/>
       </rPr>
-      <t>STONE OF DZIVOGON</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Czcionka tekstu podstawowego"/>
-        <family val="2"/>
-        <charset val="238"/>
-      </rPr>
-      <t xml:space="preserve"> id:50 oraz </t>
+      <t>SHIELD_STONE_OF_DZIVOGON</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve"> oraz </t>
     </r>
     <r>
       <rPr>
@@ -270,23 +571,24 @@
         <rFont val="Czcionka tekstu podstawowego"/>
         <charset val="238"/>
       </rPr>
-      <t>BONDCUTTER</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Czcionka tekstu podstawowego"/>
-        <family val="2"/>
-        <charset val="238"/>
-      </rPr>
-      <t xml:space="preserve"> konieczny w 33)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">19
-FOREST_1
+      <t>ITEM_BONDCUTTER</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Czcionka tekstu podstawowego"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve"> 
+konieczny w 33)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">30
+MELT_SWAMP
 </t>
     </r>
     <r>
@@ -296,244 +598,7 @@
         <rFont val="Czcionka tekstu podstawowego"/>
         <charset val="238"/>
       </rPr>
-      <t>BIES HP 6, DEF 2 ATT 2</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">9
-LAKE
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Czcionka tekstu podstawowego"/>
-        <charset val="238"/>
-      </rPr>
-      <t>DROWNER HP 5 DEF 3 ATT 5</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Czcionka tekstu podstawowego"/>
-        <family val="2"/>
-        <charset val="238"/>
-      </rPr>
-      <t xml:space="preserve">
-(po pokonaniu potwora wypada pochodnia - </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="3" tint="0.39997558519241921"/>
-        <rFont val="Czcionka tekstu podstawowego"/>
-        <charset val="238"/>
-      </rPr>
-      <t>TORCH</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Czcionka tekstu podstawowego"/>
-        <family val="2"/>
-        <charset val="238"/>
-      </rPr>
-      <t xml:space="preserve"> id:0)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">16
-MOUND_INSIDE
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Czcionka tekstu podstawowego"/>
-        <charset val="238"/>
-      </rPr>
-      <t>NIGHT PREACHER HP 20, DEF 9, ATT 8</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Czcionka tekstu podstawowego"/>
-        <family val="2"/>
-        <charset val="238"/>
-      </rPr>
-      <t xml:space="preserve"> (po pokonaniu potwora wypada </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="9" tint="-0.249977111117893"/>
-        <rFont val="Czcionka tekstu podstawowego"/>
-        <charset val="238"/>
-      </rPr>
-      <t>HEAD_SOUTHERN_SUN</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Czcionka tekstu podstawowego"/>
-        <family val="2"/>
-        <charset val="238"/>
-      </rPr>
-      <t>)
-potrzeba pochodni, żeby przejść E</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">26
-SPRING
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Czcionka tekstu podstawowego"/>
-        <charset val="238"/>
-      </rPr>
-      <t>STRIGA HP 9 DEF 5 ATT 9</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Czcionka tekstu podstawowego"/>
-        <family val="2"/>
-        <charset val="238"/>
-      </rPr>
-      <t xml:space="preserve">
-(po pokonaniu potwora wypada </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="3" tint="0.39997558519241921"/>
-        <rFont val="Czcionka tekstu podstawowego"/>
-        <charset val="238"/>
-      </rPr>
-      <t>POTION</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Czcionka tekstu podstawowego"/>
-        <family val="2"/>
-        <charset val="238"/>
-      </rPr>
-      <t xml:space="preserve"> i pozwala przejść do E)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">32
-SVAROG_STONE_CIRCLE
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Czcionka tekstu podstawowego"/>
-        <charset val="238"/>
-      </rPr>
-      <t>LESHY HP 15 DEF 4 ATT 8</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Czcionka tekstu podstawowego"/>
-        <family val="2"/>
-        <charset val="238"/>
-      </rPr>
-      <t xml:space="preserve">
-(po pokonaniu potwora wypada kamień do broni - </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="9" tint="-0.249977111117893"/>
-        <rFont val="Czcionka tekstu podstawowego"/>
-        <charset val="238"/>
-      </rPr>
-      <t>BRONZE STONE</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Czcionka tekstu podstawowego"/>
-        <family val="2"/>
-        <charset val="238"/>
-      </rPr>
-      <t xml:space="preserve"> id:40)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">21
-CAVE
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="9" tint="-0.249977111117893"/>
-        <rFont val="Czcionka tekstu podstawowego"/>
-        <charset val="238"/>
-      </rPr>
-      <t>BLOOD_HARVEST (ATT +3)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Czcionka tekstu podstawowego"/>
-        <family val="2"/>
-        <charset val="238"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Czcionka tekstu podstawowego"/>
-        <charset val="238"/>
-      </rPr>
-      <t>PERUN'S STONE</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">28
-LOCATION_MORANA_CIRCLE
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Czcionka tekstu podstawowego"/>
-        <charset val="238"/>
-      </rPr>
-      <t>MORANA HP 15 DEF 7 ATT 6</t>
+      <t>KING OF DROWNERS HP 25, DEF 11, ATT 11</t>
     </r>
     <r>
       <rPr>
@@ -554,7 +619,7 @@
         <rFont val="Czcionka tekstu podstawowego"/>
         <charset val="238"/>
       </rPr>
-      <t>SVAROG'S HAMMER</t>
+      <t>DAZHBOGS DIAMOND</t>
     </r>
     <r>
       <rPr>
@@ -573,7 +638,7 @@
         <rFont val="Czcionka tekstu podstawowego"/>
         <charset val="238"/>
       </rPr>
-      <t>IRON_STRONGOLD</t>
+      <t>WEAPON_PERUNS_FLASH</t>
     </r>
     <r>
       <rPr>
@@ -585,6 +650,19 @@
       </rPr>
       <t>)</t>
     </r>
+  </si>
+  <si>
+    <t>24
+FINAL_BATTLE</t>
+  </si>
+  <si>
+    <t>7
+STONE_THRESHOLD
+(do E można przejść tylko, jeśli zdobyło się trzy artefakty)</t>
+  </si>
+  <si>
+    <t>8
+SOUNDLESS_PASS</t>
   </si>
 </sst>
 </file>
@@ -633,7 +711,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -751,11 +829,68 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -766,9 +901,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -791,6 +923,33 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1095,122 +1254,122 @@
   <sheetData>
     <row r="1" spans="1:6" ht="105.75" customHeight="1" thickBot="1">
       <c r="A1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B1" s="4">
+        <v>23</v>
+      </c>
+      <c r="B1" s="19">
         <v>2</v>
       </c>
-      <c r="C1" s="4">
+      <c r="C1" s="18">
         <v>3</v>
       </c>
-      <c r="D1" s="4">
+      <c r="D1" s="18">
         <v>4</v>
       </c>
-      <c r="E1" s="4">
+      <c r="E1" s="15">
         <v>5</v>
       </c>
-      <c r="F1" s="4">
+      <c r="F1" s="12">
         <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="99.95" customHeight="1" thickBot="1">
       <c r="A2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="4">
-        <v>8</v>
+        <v>26</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>27</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D2" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2" s="4">
+        <v>17</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" s="17">
         <v>11</v>
       </c>
-      <c r="F2" s="4">
+      <c r="F2" s="16">
         <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="99.95" customHeight="1" thickBot="1">
-      <c r="A3" s="5" t="s">
-        <v>11</v>
+      <c r="A3" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="8" t="s">
-        <v>14</v>
+      <c r="C3" s="7" t="s">
+        <v>22</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="E3" s="12" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" s="4">
+        <v>11</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" s="14">
         <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="99.95" customHeight="1" thickBot="1">
       <c r="A4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="9" t="s">
-        <v>23</v>
+      <c r="C4" s="8" t="s">
+        <v>12</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4" s="4">
-        <v>24</v>
+        <v>20</v>
+      </c>
+      <c r="F4" s="20" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="99.95" customHeight="1" thickBot="1">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="13" t="s">
         <v>24</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F5" s="4">
-        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="99.95" customHeight="1" thickBot="1">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="C6" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" s="11" t="s">
+      <c r="B6" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="7" t="s">
         <v>9</v>
-      </c>
-      <c r="F6" s="12" t="s">
-        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>